<commit_message>
updated the code Seperated the Make transfer page
</commit_message>
<xml_diff>
--- a/src/main/resources/Testdata/Login.xlsx
+++ b/src/main/resources/Testdata/Login.xlsx
@@ -25,14 +25,14 @@
     <t>Testuser98</t>
   </si>
   <si>
-    <t>Test#123</t>
+    <t>Test@123</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -44,6 +44,13 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,14 +75,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -372,7 +385,7 @@
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -387,11 +400,14 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated the code Beneficiary details page hardcodd vaues are changed to dynamic
</commit_message>
<xml_diff>
--- a/src/main/resources/Testdata/Login.xlsx
+++ b/src/main/resources/Testdata/Login.xlsx
@@ -22,10 +22,10 @@
     <t>password</t>
   </si>
   <si>
-    <t>Testuser98</t>
+    <t>PoojaAmin</t>
   </si>
   <si>
-    <t>Test@123</t>
+    <t>Admin@2020</t>
   </si>
 </sst>
 </file>
@@ -384,7 +384,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
     <col min="2" max="2" width="39.109375" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>